<commit_message>
docs: add accessibility defect documentation
</commit_message>
<xml_diff>
--- a/SauceDemo_Test_Cases.xlsx
+++ b/SauceDemo_Test_Cases.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\SwagLabs_Playwright_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843E2E85-EE13-49D7-A38E-D3A4ECB3179E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D49371-2864-4904-8B73-67A3542CFB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="1260" windowWidth="13860" windowHeight="11700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="13860" windowHeight="11700" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
     <sheet name="Test Summary" sheetId="2" r:id="rId2"/>
     <sheet name="Automation Traceability" sheetId="3" r:id="rId3"/>
+    <sheet name="Accessibility Defects" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$K$35</definedName>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="247">
   <si>
     <t>TC ID</t>
   </si>
@@ -613,13 +614,166 @@
   </si>
   <si>
     <t>tests/checkout.spec.ts + tests/checkout-negative.spec.ts</t>
+  </si>
+  <si>
+    <t>A11Y-001</t>
+  </si>
+  <si>
+    <t>Accessibility</t>
+  </si>
+  <si>
+    <t>Scan Login page for accessibility violations</t>
+  </si>
+  <si>
+    <t>Application is available and Login page is open</t>
+  </si>
+  <si>
+    <t>1. Open Login page. 2. Run Axe accessibility scan. 3. Review detected violations.</t>
+  </si>
+  <si>
+    <t>Login page</t>
+  </si>
+  <si>
+    <t>Axe scan identifies and reports any accessibility violations found on the Login page.</t>
+  </si>
+  <si>
+    <t>A11Y-002</t>
+  </si>
+  <si>
+    <t>Scan Products page for accessibility violations</t>
+  </si>
+  <si>
+    <t>User is logged in and Products page is displayed</t>
+  </si>
+  <si>
+    <t>1. Login with valid credentials. 2. Navigate to Products page. 3. Run Axe accessibility scan. 4. Review detected violations.</t>
+  </si>
+  <si>
+    <t>Valid SauceDemo credentials</t>
+  </si>
+  <si>
+    <t>Axe scan identifies and reports any accessibility violations found on the Products page.</t>
+  </si>
+  <si>
+    <t>A11Y-003</t>
+  </si>
+  <si>
+    <t>Scan Cart page for accessibility violations</t>
+  </si>
+  <si>
+    <t>User is logged in and at least one product is added to the cart</t>
+  </si>
+  <si>
+    <t>1. Login with valid credentials. 2. Add Sauce Labs Backpack to cart. 3. Open Cart page. 4. Run Axe accessibility scan. 5. Review detected violations.</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Axe scan identifies and reports any accessibility violations found on the Cart page.</t>
+  </si>
+  <si>
+    <t>A11Y-004</t>
+  </si>
+  <si>
+    <t>Scan Checkout page for accessibility violations</t>
+  </si>
+  <si>
+    <t>User is logged in and has a product in the cart</t>
+  </si>
+  <si>
+    <t>1. Login with valid credentials. 2. Add Sauce Labs Backpack to cart. 3. Open Cart. 4. Click Checkout. 5. Enter customer information. 6. Continue to Overview. 7. Run Axe accessibility scan. 8. Review detected violations.</t>
+  </si>
+  <si>
+    <t>Aya Hesham, 12345</t>
+  </si>
+  <si>
+    <t>Axe scan identifies and reports any accessibility violations found on the Checkout page.</t>
+  </si>
+  <si>
+    <t>Updated Test Coverage</t>
+  </si>
+  <si>
+    <t>Total documented test cases</t>
+  </si>
+  <si>
+    <t>Functional test cases</t>
+  </si>
+  <si>
+    <t>Accessibility test cases</t>
+  </si>
+  <si>
+    <t>Defect ID</t>
+  </si>
+  <si>
+    <t>Page</t>
+  </si>
+  <si>
+    <t>Axe Rule</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Affected Elements</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Browsers</t>
+  </si>
+  <si>
+    <t>AD-001</t>
+  </si>
+  <si>
+    <t>landmark-one-main</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>Document does not have a main landmark</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Chromium, Firefox, WebKit</t>
+  </si>
+  <si>
+    <t>AD-002</t>
+  </si>
+  <si>
+    <t>page-has-heading-one</t>
+  </si>
+  <si>
+    <t>Page does not contain a level-one heading</t>
+  </si>
+  <si>
+    <t>AD-003</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>Some page content is not contained by landmarks</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -633,8 +787,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,6 +803,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -668,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -683,6 +847,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -985,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2167,6 +2338,190 @@
         <v>45</v>
       </c>
     </row>
+    <row r="36" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="6"/>
+    </row>
+    <row r="37" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K37" s="6"/>
+    </row>
+    <row r="38" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K38" s="6"/>
+    </row>
+    <row r="39" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K39" s="6"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K35" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2175,7 +2530,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2235,8 +2590,33 @@
       <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B9">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>224</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2311,4 +2691,128 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A3E6A85-BA95-4A95-B89C-3092F7CC35C9}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>